<commit_message>
Atualiza dados do Smart Stock3
</commit_message>
<xml_diff>
--- a/data-source/estoque.xlsx
+++ b/data-source/estoque.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\impre\OneDrive\Área de Trabalho\prompt-smart-stock-sight (4) (1)antig\data-source\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b319cc1648f3add/Área de Trabalho/prompt-smart-stock-sight (4) (1)antig/data-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{53463D38-B808-4614-9B2C-7C4C4AD7B330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{53463D38-B808-4614-9B2C-7C4C4AD7B330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0805019-D2E7-4627-9423-52FDE4358B82}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8547,7 +8547,7 @@
         <v>170</v>
       </c>
       <c r="D161" s="4">
-        <v>338</v>
+        <v>643</v>
       </c>
       <c r="E161" s="3" t="s">
         <v>13</v>

</xml_diff>